<commit_message>
Refactor: unify application and form input types - Preserve the role field and existing application statuses - Separate creation input and status filter types from application records - Use shared types across components and mock data
</commit_message>
<xml_diff>
--- a/Docs/JobTracker_Development_Tasks.xlsx
+++ b/Docs/JobTracker_Development_Tasks.xlsx
@@ -5,23 +5,34 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Develop\Projects\FrontEnd\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Develop\Projects\FrontEnd\job-tracker-fullStack\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49F1F79F-0F0F-425F-BE63-28E60B96C2B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0382327F-3555-4769-9478-D9C93A5102C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9045" yWindow="2040" windowWidth="28035" windowHeight="16950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="任务进度" sheetId="1" r:id="rId1"/>
     <sheet name="需求详情" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="385">
   <si>
     <t>Job Tracker 开发任务进度</t>
   </si>
@@ -98,9 +109,6 @@
     <t>统一申请和输入类型</t>
   </si>
   <si>
-    <t>正在梳理公共类型；mock 提取方案已讨论，尚未确认完成</t>
-  </si>
-  <si>
     <t>S1-02</t>
   </si>
   <si>
@@ -444,9 +452,6 @@
   </si>
   <si>
     <t>任务类型</t>
-  </si>
-  <si>
-    <t>package.json 锁文件 README</t>
   </si>
   <si>
     <t>恢复一个可继续开发的本地基线。</t>
@@ -487,11 +492,6 @@
   </si>
   <si>
     <t>表单、卡片和列表使用一致字段。</t>
-  </si>
-  <si>
-    <t>1. 检查 Application 字段；保留 role 和现有合法状态。
-2. 补齐五种状态联合类型，区分输入类型与完整记录。
-3. 让 Card、Form、FilterBar 引用公共类型并修复 mock。</t>
   </si>
   <si>
     <t>必要类型检查通过；不存在 position 与 role 混用。</t>
@@ -1280,6 +1280,271 @@
     <t>任务记录已建立；已有功能操作和真实目录待复核</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>组件抽离</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>+mock
+2.build task records</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026.10.4</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">package.json </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>锁文件</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> README</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>复核</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>检查</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Application </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>字段；保留</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> role </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">和现有合法状态。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">补齐五种状态联合类型，区分输入类型与完整记录。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>让</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Card</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Form</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">FilterBar </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>引用公共类型并修复</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> mock</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>。</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026.10.9</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>完成验收1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>npx tsc --noEmit 2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>新增删除功能验证</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -1288,7 +1553,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1340,6 +1605,39 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF223449"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF223449"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF223449"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF223449"/>
+      <name val="DengXian"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF223449"/>
+      <name val="Noto Sans CJK SC"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1377,7 +1675,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1427,48 +1725,18 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="18">
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1535,6 +1803,42 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1549,28 +1853,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="JobTrackerTasks" displayName="JobTrackerTasks" ref="A7:K52" totalsRowShown="0" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="JobTrackerTasks" displayName="JobTrackerTasks" ref="A7:K52" totalsRowShown="0" dataDxfId="17">
   <autoFilter ref="A7:K52" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="顺序" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="阶段" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="任务编号" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="任务名称" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="任务状态" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="前置依赖" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="验收结果" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Git 提交" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="完成日期" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="剩余问题" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="当前进度依据" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="顺序" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="阶段" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="任务编号" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="任务名称" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="任务状态" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="前置依赖" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="验收结果" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Git 提交" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="完成日期" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="剩余问题" dataDxfId="7"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="当前进度依据" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="JobTrackerDetails" displayName="JobTrackerDetails" ref="A7:H52" totalsRowShown="0">
-  <autoFilter ref="A7:H52" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="JobTrackerDetails" displayName="JobTrackerDetails" ref="A5:H50" totalsRowShown="0">
+  <autoFilter ref="A5:H50" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="任务编号"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="任务名称"/>
@@ -1870,14 +2174,14 @@
       </c>
       <c r="D5" s="4">
         <f>COUNTIFS(E8:E52,"已验收")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="5">
         <f>D5/B5</f>
-        <v>4.4444444444444446E-2</v>
+        <v>6.6666666666666666E-2</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>6</v>
@@ -1891,7 +2195,7 @@
       </c>
       <c r="J5" s="4">
         <f>COUNTIFS(E8:E52,"待复核")</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K5" s="4"/>
     </row>
@@ -1928,16 +2232,16 @@
         <v>13</v>
       </c>
       <c r="G7" s="15" t="s">
+        <v>369</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="J7" s="15" t="s">
         <v>372</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>373</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>374</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>375</v>
       </c>
       <c r="K7" s="6" t="s">
         <v>14</v>
@@ -1963,19 +2267,19 @@
         <v>18</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="44.1" customHeight="1">
@@ -1998,15 +2302,19 @@
         <v>16</v>
       </c>
       <c r="G9" s="16" t="s">
+        <v>373</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>379</v>
+      </c>
+      <c r="J9" s="16" t="s">
         <v>376</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="16" t="s">
-        <v>379</v>
-      </c>
       <c r="K9" s="14" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="44.1" customHeight="1">
@@ -2023,17 +2331,21 @@
         <v>24</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="8"/>
+      <c r="G10" s="16" t="s">
+        <v>373</v>
+      </c>
       <c r="H10" s="8"/>
-      <c r="I10" s="9"/>
+      <c r="I10" s="9" t="s">
+        <v>383</v>
+      </c>
       <c r="J10" s="8"/>
-      <c r="K10" s="7" t="s">
-        <v>25</v>
+      <c r="K10" s="18" t="s">
+        <v>384</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="42" customHeight="1">
@@ -2044,10 +2356,10 @@
         <v>22</v>
       </c>
       <c r="C11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>26</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>27</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>6</v>
@@ -2060,7 +2372,7 @@
       <c r="I11" s="9"/>
       <c r="J11" s="8"/>
       <c r="K11" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="42" customHeight="1">
@@ -2071,16 +2383,16 @@
         <v>22</v>
       </c>
       <c r="C12" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>30</v>
-      </c>
       <c r="E12" s="8" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
@@ -2098,16 +2410,16 @@
         <v>22</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>32</v>
-      </c>
       <c r="E13" s="8" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
@@ -2125,16 +2437,16 @@
         <v>22</v>
       </c>
       <c r="C14" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="7" t="s">
-        <v>34</v>
-      </c>
       <c r="E14" s="8" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
@@ -2152,16 +2464,16 @@
         <v>22</v>
       </c>
       <c r="C15" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>36</v>
-      </c>
       <c r="E15" s="8" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
@@ -2179,16 +2491,16 @@
         <v>22</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>38</v>
-      </c>
       <c r="E16" s="8" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -2206,16 +2518,16 @@
         <v>22</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="E17" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>41</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
@@ -2230,26 +2542,26 @@
         <v>11</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="E18" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>45</v>
-      </c>
       <c r="F18" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="9"/>
       <c r="J18" s="8"/>
       <c r="K18" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="42" customHeight="1">
@@ -2257,26 +2569,26 @@
         <v>12</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>43</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="9"/>
       <c r="J19" s="8"/>
       <c r="K19" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="42" customHeight="1">
@@ -2284,26 +2596,26 @@
         <v>13</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F20" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>43</v>
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="9"/>
       <c r="J20" s="8"/>
       <c r="K20" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="42" customHeight="1">
@@ -2311,26 +2623,26 @@
         <v>14</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C21" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="E21" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F21" s="8" t="s">
         <v>52</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>53</v>
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="9"/>
       <c r="J21" s="8"/>
       <c r="K21" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="42" customHeight="1">
@@ -2338,26 +2650,26 @@
         <v>15</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D22" s="7" t="s">
-        <v>55</v>
-      </c>
       <c r="E22" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
       <c r="I22" s="9"/>
       <c r="J22" s="8"/>
       <c r="K22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="42" customHeight="1">
@@ -2365,26 +2677,26 @@
         <v>16</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C23" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="E23" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F23" s="8" t="s">
         <v>57</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>58</v>
       </c>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
       <c r="I23" s="9"/>
       <c r="J23" s="8"/>
       <c r="K23" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="42" customHeight="1">
@@ -2392,26 +2704,26 @@
         <v>17</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="D24" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="7" t="s">
-        <v>61</v>
-      </c>
       <c r="E24" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="9"/>
       <c r="J24" s="8"/>
       <c r="K24" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="42" customHeight="1">
@@ -2419,26 +2731,26 @@
         <v>18</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F25" s="8" t="s">
         <v>59</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>60</v>
       </c>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
       <c r="J25" s="8"/>
       <c r="K25" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="42" customHeight="1">
@@ -2446,26 +2758,26 @@
         <v>19</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C26" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="E26" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F26" s="8" t="s">
         <v>65</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>66</v>
       </c>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
       <c r="J26" s="8"/>
       <c r="K26" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="42" customHeight="1">
@@ -2473,26 +2785,26 @@
         <v>20</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C27" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="7" t="s">
-        <v>68</v>
-      </c>
       <c r="E27" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
       <c r="J27" s="8"/>
       <c r="K27" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="42" customHeight="1">
@@ -2500,26 +2812,26 @@
         <v>21</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C28" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="E28" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F28" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>71</v>
       </c>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
       <c r="J28" s="8"/>
       <c r="K28" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="42" customHeight="1">
@@ -2527,26 +2839,26 @@
         <v>22</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C29" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D29" s="7" t="s">
-        <v>73</v>
-      </c>
       <c r="E29" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G29" s="8"/>
       <c r="H29" s="8"/>
       <c r="I29" s="9"/>
       <c r="J29" s="8"/>
       <c r="K29" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="42" customHeight="1">
@@ -2554,26 +2866,26 @@
         <v>23</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C30" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="E30" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F30" s="8" t="s">
         <v>75</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>76</v>
       </c>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
       <c r="I30" s="9"/>
       <c r="J30" s="8"/>
       <c r="K30" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="42" customHeight="1">
@@ -2581,26 +2893,26 @@
         <v>24</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="D31" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="D31" s="7" t="s">
-        <v>79</v>
-      </c>
       <c r="E31" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
       <c r="I31" s="9"/>
       <c r="J31" s="8"/>
       <c r="K31" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="42" customHeight="1">
@@ -2608,26 +2920,26 @@
         <v>25</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F32" s="8" t="s">
         <v>77</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>78</v>
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
       <c r="I32" s="9"/>
       <c r="J32" s="8"/>
       <c r="K32" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="42" customHeight="1">
@@ -2635,26 +2947,26 @@
         <v>26</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C33" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D33" s="7" t="s">
-        <v>83</v>
-      </c>
       <c r="E33" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
       <c r="I33" s="9"/>
       <c r="J33" s="8"/>
       <c r="K33" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="42" customHeight="1">
@@ -2662,26 +2974,26 @@
         <v>27</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C34" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D34" s="7" t="s">
-        <v>85</v>
-      </c>
       <c r="E34" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
       <c r="I34" s="9"/>
       <c r="J34" s="8"/>
       <c r="K34" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="42" customHeight="1">
@@ -2689,26 +3001,26 @@
         <v>28</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C35" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>87</v>
-      </c>
       <c r="E35" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
       <c r="I35" s="9"/>
       <c r="J35" s="8"/>
       <c r="K35" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="42" customHeight="1">
@@ -2716,26 +3028,26 @@
         <v>29</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C36" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D36" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="E36" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F36" s="8" t="s">
         <v>89</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F36" s="8" t="s">
-        <v>90</v>
       </c>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
       <c r="I36" s="9"/>
       <c r="J36" s="8"/>
       <c r="K36" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="42" customHeight="1">
@@ -2743,26 +3055,26 @@
         <v>30</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C37" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D37" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D37" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="E37" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G37" s="8"/>
       <c r="H37" s="8"/>
       <c r="I37" s="9"/>
       <c r="J37" s="8"/>
       <c r="K37" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="42" customHeight="1">
@@ -2770,26 +3082,26 @@
         <v>31</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C38" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D38" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="E38" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F38" s="8" t="s">
         <v>94</v>
-      </c>
-      <c r="E38" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>95</v>
       </c>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
       <c r="I38" s="9"/>
       <c r="J38" s="8"/>
       <c r="K38" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="42" customHeight="1">
@@ -2797,26 +3109,26 @@
         <v>32</v>
       </c>
       <c r="B39" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C39" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="D39" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="D39" s="7" t="s">
-        <v>98</v>
-      </c>
       <c r="E39" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G39" s="8"/>
       <c r="H39" s="8"/>
       <c r="I39" s="9"/>
       <c r="J39" s="8"/>
       <c r="K39" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="42" customHeight="1">
@@ -2824,26 +3136,26 @@
         <v>33</v>
       </c>
       <c r="B40" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F40" s="8" t="s">
         <v>96</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F40" s="8" t="s">
-        <v>97</v>
       </c>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
       <c r="I40" s="9"/>
       <c r="J40" s="8"/>
       <c r="K40" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="42" customHeight="1">
@@ -2851,26 +3163,26 @@
         <v>34</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C41" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D41" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="D41" s="7" t="s">
-        <v>102</v>
-      </c>
       <c r="E41" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
       <c r="I41" s="9"/>
       <c r="J41" s="8"/>
       <c r="K41" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="42" customHeight="1">
@@ -2878,26 +3190,26 @@
         <v>35</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C42" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D42" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="E42" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F42" s="8" t="s">
         <v>104</v>
-      </c>
-      <c r="E42" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F42" s="8" t="s">
-        <v>105</v>
       </c>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
       <c r="I42" s="9"/>
       <c r="J42" s="8"/>
       <c r="K42" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="42" customHeight="1">
@@ -2905,26 +3217,26 @@
         <v>36</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C43" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D43" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D43" s="7" t="s">
-        <v>107</v>
-      </c>
       <c r="E43" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G43" s="8"/>
       <c r="H43" s="8"/>
       <c r="I43" s="9"/>
       <c r="J43" s="8"/>
       <c r="K43" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="42" customHeight="1">
@@ -2932,26 +3244,26 @@
         <v>37</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C44" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D44" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="D44" s="7" t="s">
-        <v>109</v>
-      </c>
       <c r="E44" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
       <c r="I44" s="9"/>
       <c r="J44" s="8"/>
       <c r="K44" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="42" customHeight="1">
@@ -2959,26 +3271,26 @@
         <v>38</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C45" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D45" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D45" s="7" t="s">
-        <v>111</v>
-      </c>
       <c r="E45" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G45" s="8"/>
       <c r="H45" s="8"/>
       <c r="I45" s="9"/>
       <c r="J45" s="8"/>
       <c r="K45" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="42" customHeight="1">
@@ -2986,26 +3298,26 @@
         <v>39</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C46" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D46" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="E46" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F46" s="8" t="s">
         <v>113</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F46" s="8" t="s">
-        <v>114</v>
       </c>
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
       <c r="I46" s="9"/>
       <c r="J46" s="8"/>
       <c r="K46" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="42" customHeight="1">
@@ -3013,26 +3325,26 @@
         <v>40</v>
       </c>
       <c r="B47" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C47" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="D47" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D47" s="7" t="s">
+      <c r="E47" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F47" s="8" t="s">
         <v>117</v>
-      </c>
-      <c r="E47" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F47" s="8" t="s">
-        <v>118</v>
       </c>
       <c r="G47" s="8"/>
       <c r="H47" s="8"/>
       <c r="I47" s="9"/>
       <c r="J47" s="8"/>
       <c r="K47" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="42" customHeight="1">
@@ -3040,26 +3352,26 @@
         <v>41</v>
       </c>
       <c r="B48" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="E48" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F48" s="8" t="s">
         <v>115</v>
-      </c>
-      <c r="C48" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D48" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E48" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F48" s="8" t="s">
-        <v>116</v>
       </c>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
       <c r="I48" s="9"/>
       <c r="J48" s="8"/>
       <c r="K48" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="42" customHeight="1">
@@ -3067,26 +3379,26 @@
         <v>42</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C49" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D49" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D49" s="7" t="s">
-        <v>122</v>
-      </c>
       <c r="E49" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
       <c r="I49" s="9"/>
       <c r="J49" s="8"/>
       <c r="K49" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="42" customHeight="1">
@@ -3094,26 +3406,26 @@
         <v>43</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C50" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D50" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D50" s="7" t="s">
-        <v>124</v>
-      </c>
       <c r="E50" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
       <c r="I50" s="9"/>
       <c r="J50" s="8"/>
       <c r="K50" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="42" customHeight="1">
@@ -3121,26 +3433,26 @@
         <v>44</v>
       </c>
       <c r="B51" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="C51" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="D51" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="D51" s="7" t="s">
+      <c r="E51" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="E51" s="8" t="s">
-        <v>128</v>
-      </c>
       <c r="F51" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
       <c r="I51" s="9"/>
       <c r="J51" s="8"/>
       <c r="K51" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="42" customHeight="1">
@@ -3148,47 +3460,47 @@
         <v>45</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C52" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D52" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="D52" s="7" t="s">
-        <v>131</v>
-      </c>
       <c r="E52" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="9"/>
       <c r="J52" s="8"/>
       <c r="K52" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <conditionalFormatting sqref="E8:E52">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>$E8="未开始"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>$E8="待复核"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>$E8="开发中"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>$E8="待验收"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>$E8="已验收"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="6">
+    <cfRule type="expression" dxfId="0" priority="6">
       <formula>$E8="暂缓"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3209,15 +3521,15 @@
   <sheetPr>
     <tabColor rgb="FF7E91A5"/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="26.875" customWidth="1"/>
-    <col min="3" max="3" width="44" customWidth="1"/>
-    <col min="4" max="4" width="35.25" customWidth="1"/>
-    <col min="5" max="5" width="58.625" customWidth="1"/>
-    <col min="6" max="6" width="53.5" customWidth="1"/>
+    <col min="3" max="3" width="34.875" customWidth="1"/>
+    <col min="4" max="4" width="34.125" customWidth="1"/>
+    <col min="5" max="5" width="54.25" customWidth="1"/>
+    <col min="6" max="6" width="28.25" customWidth="1"/>
     <col min="7" max="7" width="26.375" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
   </cols>
@@ -3234,7 +3546,7 @@
     </row>
     <row r="2" spans="1:8" ht="27.95" customHeight="1">
       <c r="A2" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -3246,7 +3558,7 @@
     </row>
     <row r="3" spans="1:8" ht="24" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
@@ -3258,7 +3570,7 @@
     </row>
     <row r="4" spans="1:8" ht="24" customHeight="1">
       <c r="A4" s="12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -3268,1220 +3580,1200 @@
       <c r="G4" s="12"/>
       <c r="H4" s="12"/>
     </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-    </row>
-    <row r="7" spans="1:8" ht="30" customHeight="1">
-      <c r="A7" s="6" t="s">
+    <row r="5" spans="1:8" ht="30" customHeight="1">
+      <c r="A5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C5" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="H7" s="6" t="s">
+    </row>
+    <row r="6" spans="1:8" ht="68.099999999999994" customHeight="1">
+      <c r="A6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>380</v>
+      </c>
+      <c r="D6" s="13" t="s">
         <v>140</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="68.099999999999994" customHeight="1">
+      <c r="A7" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A8" s="13" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>143</v>
+        <v>382</v>
       </c>
       <c r="F8" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="H8" s="13" t="s">
         <v>144</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="H8" s="13" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A10" s="13" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A11" s="13" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A13" s="13" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A14" s="13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A16" s="13" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A17" s="13" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>146</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A18" s="13" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E18" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="G18" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="H18" s="13" t="s">
         <v>195</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="H18" s="13" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A19" s="13" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A20" s="13" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A22" s="13" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A23" s="13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A24" s="13" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A26" s="13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A27" s="13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A28" s="13" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A30" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A31" s="13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="G31" s="13" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A32" s="13" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A33" s="13" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A34" s="13" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A36" s="13" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A37" s="13" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A38" s="13" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="G38" s="13" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="68.099999999999994" customHeight="1">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="78" customHeight="1">
       <c r="A39" s="13" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="F39" s="13" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="G39" s="13" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A40" s="13" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="G40" s="13" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="78" customHeight="1">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A41" s="13" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="G41" s="13" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A42" s="13" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="G42" s="13" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="68.099999999999994" customHeight="1">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="78" customHeight="1">
       <c r="A43" s="13" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="G43" s="13" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="H43" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A44" s="13" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="F44" s="13" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="G44" s="13" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="H44" s="13" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" ht="78" customHeight="1">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A45" s="13" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A46" s="13" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="G46" s="13" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="H46" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A47" s="13" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="G47" s="13" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A48" s="13" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="F48" s="13" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="G48" s="13" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="H48" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A49" s="13" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="G49" s="13" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="H49" s="13" t="s">
-        <v>198</v>
+        <v>361</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A50" s="13" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="F50" s="13" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="G50" s="13" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="H50" s="13" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" ht="68.099999999999994" customHeight="1">
-      <c r="A51" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="B51" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="C51" s="13" t="s">
-        <v>359</v>
-      </c>
-      <c r="D51" s="13" t="s">
-        <v>360</v>
-      </c>
-      <c r="E51" s="13" t="s">
         <v>361</v>
-      </c>
-      <c r="F51" s="13" t="s">
-        <v>362</v>
-      </c>
-      <c r="G51" s="13" t="s">
-        <v>363</v>
-      </c>
-      <c r="H51" s="13" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" ht="68.099999999999994" customHeight="1">
-      <c r="A52" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="B52" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="C52" s="13" t="s">
-        <v>365</v>
-      </c>
-      <c r="D52" s="13" t="s">
-        <v>366</v>
-      </c>
-      <c r="E52" s="13" t="s">
-        <v>367</v>
-      </c>
-      <c r="F52" s="13" t="s">
-        <v>368</v>
-      </c>
-      <c r="G52" s="13" t="s">
-        <v>369</v>
-      </c>
-      <c r="H52" s="13" t="s">
-        <v>364</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S0-03 refactor: migrate UI styles to SCSS and organize applications layout
</commit_message>
<xml_diff>
--- a/Docs/JobTracker_Development_Tasks.xlsx
+++ b/Docs/JobTracker_Development_Tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Develop\Projects\FrontEnd\job-tracker-fullStack\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0382327F-3555-4769-9478-D9C93A5102C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDCE5EBF-521F-4A91-AF92-CD5EDD72BEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9045" yWindow="2040" windowWidth="28035" windowHeight="16950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="386">
   <si>
     <t>Job Tracker 开发任务进度</t>
   </si>
@@ -1543,6 +1543,13 @@
       </rPr>
       <t>新增删除功能验证</t>
     </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Refactor: unify application and form input types
+- Preserve the role field and existing application statuses
+- Separate creation input and status filter types from application records
+- Use shared types across components and mock data</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -2097,7 +2104,7 @@
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="15.125" customWidth="1"/>
     <col min="7" max="7" width="10.375" customWidth="1"/>
-    <col min="8" max="8" width="30.25" customWidth="1"/>
+    <col min="8" max="8" width="36" customWidth="1"/>
     <col min="9" max="9" width="9.5" customWidth="1"/>
     <col min="10" max="10" width="19.25" customWidth="1"/>
     <col min="11" max="11" width="45" customWidth="1"/>
@@ -2317,7 +2324,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="44.1" customHeight="1">
+    <row r="10" spans="1:11" ht="122.25" customHeight="1">
       <c r="A10" s="7">
         <v>3</v>
       </c>
@@ -2339,7 +2346,9 @@
       <c r="G10" s="16" t="s">
         <v>373</v>
       </c>
-      <c r="H10" s="8"/>
+      <c r="H10" s="8" t="s">
+        <v>385</v>
+      </c>
       <c r="I10" s="9" t="s">
         <v>383</v>
       </c>

</xml_diff>

<commit_message>
S0-03 feat: add application modal and unify styles with SCSS
- Add Sass support and shared design tokens and mixins
- Migrate component styles to SCSS with BEM naming
- Move the application form into a reusable Radix UI modal
- Support form submission through the submit button and Enter key
</commit_message>
<xml_diff>
--- a/Docs/JobTracker_Development_Tasks.xlsx
+++ b/Docs/JobTracker_Development_Tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Develop\Projects\FrontEnd\job-tracker-fullStack\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDCE5EBF-521F-4A91-AF92-CD5EDD72BEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1445B38-DC1A-4275-9C71-911833993FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9045" yWindow="2040" windowWidth="28035" windowHeight="16950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9045" yWindow="2040" windowWidth="28035" windowHeight="16950" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="任务进度" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="395">
   <si>
     <t>Job Tracker 开发任务进度</t>
   </si>
@@ -58,25 +58,10 @@
     <t>待复核</t>
   </si>
   <si>
-    <t>顺序</t>
-  </si>
-  <si>
-    <t>阶段</t>
-  </si>
-  <si>
     <t>任务编号</t>
   </si>
   <si>
     <t>任务名称</t>
-  </si>
-  <si>
-    <t>任务状态</t>
-  </si>
-  <si>
-    <t>前置依赖</t>
-  </si>
-  <si>
-    <t>当前进度依据</t>
   </si>
   <si>
     <t>环境复核</t>
@@ -1228,35 +1213,6 @@
   </si>
   <si>
     <t>完成</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>验收结果</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Git </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="DengXian"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>提交</t>
-    </r>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>完成日期</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>剩余问题</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
@@ -1552,6 +1508,324 @@
 - Use shared types across components and mock data</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
+  <si>
+    <t>页面风格确认</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>S0-03</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>页面配色、交互风格、设计参考</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>S0-01</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>全面修改页面样式
+参考https://linear.app/</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">S0-03 refactor: migrate UI styles to SCSS and organize applications layout
+</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Order</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stage</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Task No.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Task</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Task status</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pre-requirement</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Result</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Git </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="3"/>
+      </rPr>
+      <t>submit</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Finish date</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Outstanding issues</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Progress</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>安装适配</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>sass</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>依赖</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Noto Sans CJK SC"/>
+      </rPr>
+      <t xml:space="preserve">
+2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>设置全局颜色到</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>global.scss</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>_token.scss</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>_mixin.scss</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>等中
+3.遍历所有组件，按</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>scss</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>方式配套层叠样式表
+4.分离</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>add application</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>到弹窗(用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>radix-ui</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>库封装</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>modal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Noto Sans CJK SC"/>
+      </rPr>
+      <t xml:space="preserve">
+5.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>修改</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>ApplicationForm</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>表单为</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>scss</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -1560,7 +1834,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1645,6 +1919,20 @@
       <family val="2"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1682,7 +1970,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1737,6 +2025,12 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1860,28 +2154,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="JobTrackerTasks" displayName="JobTrackerTasks" ref="A7:K52" totalsRowShown="0" dataDxfId="17">
-  <autoFilter ref="A7:K52" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="JobTrackerTasks" displayName="JobTrackerTasks" ref="A7:K53" totalsRowShown="0" dataDxfId="17">
+  <autoFilter ref="A7:K53" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="顺序" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="阶段" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="任务编号" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="任务名称" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="任务状态" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="前置依赖" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="验收结果" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Git 提交" dataDxfId="9"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="完成日期" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="剩余问题" dataDxfId="7"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="当前进度依据" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Stage" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Task No." dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Task" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Task status" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Pre-requirement" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Result" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Git submit" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Finish date" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Outstanding issues" dataDxfId="7"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Progress" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="JobTrackerDetails" displayName="JobTrackerDetails" ref="A5:H50" totalsRowShown="0">
-  <autoFilter ref="A5:H50" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="JobTrackerDetails" displayName="JobTrackerDetails" ref="A5:H51" totalsRowShown="0">
+  <autoFilter ref="A5:H51" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="任务编号"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="任务名称"/>
@@ -2094,10 +2388,10 @@
   <sheetPr>
     <tabColor rgb="FF243B53"/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="4.25" customWidth="1"/>
+    <col min="1" max="1" width="7.125" customWidth="1"/>
     <col min="2" max="2" width="14.25" customWidth="1"/>
     <col min="3" max="3" width="7.5" customWidth="1"/>
     <col min="4" max="4" width="25.5" customWidth="1"/>
@@ -2173,14 +2467,14 @@
         <v>3</v>
       </c>
       <c r="B5" s="4">
-        <f>COUNTA(C8:C52)</f>
-        <v>45</v>
+        <f>COUNTA(C8:C53)</f>
+        <v>46</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>4</v>
       </c>
       <c r="D5" s="4">
-        <f>COUNTIFS(E8:E52,"已验收")</f>
+        <f>COUNTIFS(E8:E53,"已验收")</f>
         <v>3</v>
       </c>
       <c r="E5" s="4" t="s">
@@ -2188,20 +2482,20 @@
       </c>
       <c r="F5" s="5">
         <f>D5/B5</f>
-        <v>6.6666666666666666E-2</v>
+        <v>6.5217391304347824E-2</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="4">
-        <f>COUNTIFS(E8:E52,"开发中")</f>
+        <f>COUNTIFS(E8:E53,"开发中")</f>
         <v>1</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="J5" s="4">
-        <f>COUNTIFS(E8:E52,"待复核")</f>
+        <f>COUNTIFS(E8:E53,"待复核")</f>
         <v>0</v>
       </c>
       <c r="K5" s="4"/>
@@ -2220,38 +2514,38 @@
       <c r="K6" s="1"/>
     </row>
     <row r="7" spans="1:11" ht="30" customHeight="1">
-      <c r="A7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>13</v>
+      <c r="A7" s="20" t="s">
+        <v>383</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>385</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>386</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>387</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>388</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>369</v>
+        <v>389</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>370</v>
+        <v>390</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>371</v>
+        <v>391</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>372</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>14</v>
+        <v>392</v>
+      </c>
+      <c r="K7" s="20" t="s">
+        <v>393</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="68.25" customHeight="1">
@@ -2259,34 +2553,34 @@
         <v>1</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>4</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>375</v>
+        <v>366</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>374</v>
+        <v>365</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="44.1" customHeight="1">
@@ -2294,34 +2588,34 @@
         <v>2</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>20</v>
-      </c>
       <c r="D9" s="7" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>4</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>16</v>
+        <v>380</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="J9" s="16" t="s">
-        <v>376</v>
+        <v>367</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="122.25" customHeight="1">
@@ -2329,1171 +2623,1198 @@
         <v>3</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>4</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>385</v>
+        <v>376</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="J10" s="8"/>
       <c r="K10" s="18" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="42" customHeight="1">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="122.25" customHeight="1">
       <c r="A11" s="7">
-        <v>4</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>22</v>
+        <v>0</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>377</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>26</v>
+        <v>378</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>379</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>6</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
+        <v>380</v>
+      </c>
+      <c r="G11" s="16"/>
+      <c r="H11" s="8" t="s">
+        <v>382</v>
+      </c>
       <c r="I11" s="9"/>
       <c r="J11" s="8"/>
-      <c r="K11" s="7" t="s">
-        <v>27</v>
-      </c>
+      <c r="K11" s="18"/>
     </row>
     <row r="12" spans="1:11" ht="42" customHeight="1">
       <c r="A12" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
       <c r="I12" s="9"/>
       <c r="J12" s="8"/>
       <c r="K12" s="7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="42" customHeight="1">
       <c r="A13" s="7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="9"/>
       <c r="J13" s="8"/>
       <c r="K13" s="7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="42" customHeight="1">
       <c r="A14" s="7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="9"/>
       <c r="J14" s="8"/>
       <c r="K14" s="7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="42" customHeight="1">
       <c r="A15" s="7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="9"/>
       <c r="J15" s="8"/>
       <c r="K15" s="7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="42" customHeight="1">
       <c r="A16" s="7">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
       <c r="I16" s="9"/>
       <c r="J16" s="8"/>
       <c r="K16" s="7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="42" customHeight="1">
       <c r="A17" s="7">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D17" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="8" t="s">
-        <v>44</v>
-      </c>
       <c r="F17" s="8" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="9"/>
       <c r="J17" s="8"/>
       <c r="K17" s="7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="42" customHeight="1">
       <c r="A18" s="7">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="9"/>
       <c r="J18" s="8"/>
       <c r="K18" s="7" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="42" customHeight="1">
       <c r="A19" s="7">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="9"/>
       <c r="J19" s="8"/>
       <c r="K19" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="42" customHeight="1">
       <c r="A20" s="7">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>48</v>
-      </c>
       <c r="D20" s="7" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="9"/>
       <c r="J20" s="8"/>
       <c r="K20" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="42" customHeight="1">
       <c r="A21" s="7">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="9"/>
       <c r="J21" s="8"/>
       <c r="K21" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="42" customHeight="1">
       <c r="A22" s="7">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
       <c r="I22" s="9"/>
       <c r="J22" s="8"/>
       <c r="K22" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="42" customHeight="1">
       <c r="A23" s="7">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
       <c r="I23" s="9"/>
       <c r="J23" s="8"/>
       <c r="K23" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="42" customHeight="1">
       <c r="A24" s="7">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="9"/>
       <c r="J24" s="8"/>
       <c r="K24" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="42" customHeight="1">
       <c r="A25" s="7">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
       <c r="J25" s="8"/>
       <c r="K25" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="42" customHeight="1">
       <c r="A26" s="7">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
       <c r="J26" s="8"/>
       <c r="K26" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="42" customHeight="1">
       <c r="A27" s="7">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B27" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C27" s="7" t="s">
-        <v>66</v>
-      </c>
       <c r="D27" s="7" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
       <c r="J27" s="8"/>
       <c r="K27" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="42" customHeight="1">
       <c r="A28" s="7">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F28" s="8" t="s">
         <v>58</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>70</v>
       </c>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
       <c r="J28" s="8"/>
       <c r="K28" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="42" customHeight="1">
       <c r="A29" s="7">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G29" s="8"/>
       <c r="H29" s="8"/>
       <c r="I29" s="9"/>
       <c r="J29" s="8"/>
       <c r="K29" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="42" customHeight="1">
       <c r="A30" s="7">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
       <c r="I30" s="9"/>
       <c r="J30" s="8"/>
       <c r="K30" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="42" customHeight="1">
       <c r="A31" s="7">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
       <c r="I31" s="9"/>
       <c r="J31" s="8"/>
       <c r="K31" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="42" customHeight="1">
       <c r="A32" s="7">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
       <c r="I32" s="9"/>
       <c r="J32" s="8"/>
       <c r="K32" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="42" customHeight="1">
       <c r="A33" s="7">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F33" s="8" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="G33" s="8"/>
       <c r="H33" s="8"/>
       <c r="I33" s="9"/>
       <c r="J33" s="8"/>
       <c r="K33" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="42" customHeight="1">
       <c r="A34" s="7">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B34" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C34" s="7" t="s">
-        <v>83</v>
-      </c>
       <c r="D34" s="7" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F34" s="8" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="G34" s="8"/>
       <c r="H34" s="8"/>
       <c r="I34" s="9"/>
       <c r="J34" s="8"/>
       <c r="K34" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="42" customHeight="1">
       <c r="A35" s="7">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B35" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F35" s="8" t="s">
         <v>76</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F35" s="8" t="s">
-        <v>79</v>
       </c>
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
       <c r="I35" s="9"/>
       <c r="J35" s="8"/>
       <c r="K35" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="42" customHeight="1">
       <c r="A36" s="7">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
       <c r="I36" s="9"/>
       <c r="J36" s="8"/>
       <c r="K36" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="42" customHeight="1">
       <c r="A37" s="7">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G37" s="8"/>
       <c r="H37" s="8"/>
       <c r="I37" s="9"/>
       <c r="J37" s="8"/>
       <c r="K37" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="42" customHeight="1">
       <c r="A38" s="7">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
       <c r="I38" s="9"/>
       <c r="J38" s="8"/>
       <c r="K38" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="42" customHeight="1">
       <c r="A39" s="7">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="G39" s="8"/>
       <c r="H39" s="8"/>
       <c r="I39" s="9"/>
       <c r="J39" s="8"/>
       <c r="K39" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="42" customHeight="1">
       <c r="A40" s="7">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
       <c r="I40" s="9"/>
       <c r="J40" s="8"/>
       <c r="K40" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="42" customHeight="1">
       <c r="A41" s="7">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="G41" s="8"/>
       <c r="H41" s="8"/>
       <c r="I41" s="9"/>
       <c r="J41" s="8"/>
       <c r="K41" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="42" customHeight="1">
       <c r="A42" s="7">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B42" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C42" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="C42" s="7" t="s">
-        <v>102</v>
-      </c>
       <c r="D42" s="7" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
       <c r="I42" s="9"/>
       <c r="J42" s="8"/>
       <c r="K42" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="42" customHeight="1">
       <c r="A43" s="7">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G43" s="8"/>
       <c r="H43" s="8"/>
       <c r="I43" s="9"/>
       <c r="J43" s="8"/>
       <c r="K43" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="42" customHeight="1">
       <c r="A44" s="7">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
       <c r="I44" s="9"/>
       <c r="J44" s="8"/>
       <c r="K44" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="42" customHeight="1">
       <c r="A45" s="7">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G45" s="8"/>
       <c r="H45" s="8"/>
       <c r="I45" s="9"/>
       <c r="J45" s="8"/>
       <c r="K45" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="42" customHeight="1">
       <c r="A46" s="7">
+        <v>38</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E46" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B46" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="C46" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="D46" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>44</v>
-      </c>
       <c r="F46" s="8" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
       <c r="I46" s="9"/>
       <c r="J46" s="8"/>
       <c r="K46" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="42" customHeight="1">
       <c r="A47" s="7">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="G47" s="8"/>
       <c r="H47" s="8"/>
       <c r="I47" s="9"/>
       <c r="J47" s="8"/>
       <c r="K47" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="42" customHeight="1">
       <c r="A48" s="7">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
       <c r="I48" s="9"/>
       <c r="J48" s="8"/>
       <c r="K48" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="42" customHeight="1">
       <c r="A49" s="7">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B49" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D49" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C49" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>121</v>
-      </c>
       <c r="E49" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
       <c r="I49" s="9"/>
       <c r="J49" s="8"/>
       <c r="K49" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="42" customHeight="1">
       <c r="A50" s="7">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
       <c r="I50" s="9"/>
       <c r="J50" s="8"/>
       <c r="K50" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="42" customHeight="1">
       <c r="A51" s="7">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>127</v>
+        <v>39</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>73</v>
+        <v>115</v>
       </c>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
       <c r="I51" s="9"/>
       <c r="J51" s="8"/>
       <c r="K51" s="7" t="s">
-        <v>128</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="42" customHeight="1">
       <c r="A52" s="7">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="D52" s="7" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>111</v>
+        <v>68</v>
       </c>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="9"/>
       <c r="J52" s="8"/>
       <c r="K52" s="7" t="s">
-        <v>128</v>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="42" customHeight="1">
+      <c r="A53" s="7">
+        <v>45</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="F53" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G53" s="8"/>
+      <c r="H53" s="8"/>
+      <c r="I53" s="9"/>
+      <c r="J53" s="8"/>
+      <c r="K53" s="7" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="E8:E52">
+  <conditionalFormatting sqref="E8:E53">
     <cfRule type="expression" dxfId="5" priority="1">
       <formula>$E8="未开始"</formula>
     </cfRule>
@@ -3514,7 +3835,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="E8:E52" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="E8:E53" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"未开始,待复核,开发中,待验收,已验收,暂缓"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3530,7 +3851,7 @@
   <sheetPr>
     <tabColor rgb="FF7E91A5"/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -3555,7 +3876,7 @@
     </row>
     <row r="2" spans="1:8" ht="27.95" customHeight="1">
       <c r="A2" s="11" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -3567,7 +3888,7 @@
     </row>
     <row r="3" spans="1:8" ht="24" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
@@ -3579,7 +3900,7 @@
     </row>
     <row r="4" spans="1:8" ht="24" customHeight="1">
       <c r="A4" s="12" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -3591,1198 +3912,1214 @@
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>134</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A6" s="13" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A7" s="13" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="68.099999999999994" customHeight="1">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="112.5" customHeight="1">
       <c r="A8" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>151</v>
-      </c>
+        <v>378</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>381</v>
+      </c>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
       <c r="E8" s="13" t="s">
-        <v>382</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="H8" s="13" t="s">
-        <v>144</v>
-      </c>
+        <v>394</v>
+      </c>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>156</v>
+        <v>373</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>159</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A10" s="13" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A11" s="13" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="H12" s="13" t="s">
-        <v>159</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A13" s="13" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A14" s="13" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="H14" s="13" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A16" s="13" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>195</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A17" s="13" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="H17" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A18" s="13" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A19" s="13" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="H19" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A20" s="13" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="H20" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="H21" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A22" s="13" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="H22" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A23" s="13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="H23" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A24" s="13" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="H25" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A26" s="13" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A27" s="13" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="H27" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A28" s="13" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="H28" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="H29" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A30" s="13" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="H30" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A31" s="13" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="G31" s="13" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A32" s="13" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A33" s="13" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="H33" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A34" s="13" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="H34" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="H35" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A36" s="13" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="H36" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A37" s="13" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A38" s="13" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C38" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="G38" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="H38" s="13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="68.099999999999994" customHeight="1">
+      <c r="A39" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>296</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>297</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="F39" s="13" t="s">
+        <v>299</v>
+      </c>
+      <c r="G39" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="H39" s="13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="78" customHeight="1">
+      <c r="A40" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="C40" s="13" t="s">
         <v>301</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D40" s="13" t="s">
         <v>302</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="E40" s="13" t="s">
         <v>303</v>
       </c>
-      <c r="F38" s="13" t="s">
+      <c r="F40" s="13" t="s">
         <v>304</v>
       </c>
-      <c r="G38" s="13" t="s">
+      <c r="G40" s="13" t="s">
         <v>305</v>
       </c>
-      <c r="H38" s="13" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="78" customHeight="1">
-      <c r="A39" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="C39" s="13" t="s">
-        <v>306</v>
-      </c>
-      <c r="D39" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="E39" s="13" t="s">
-        <v>308</v>
-      </c>
-      <c r="F39" s="13" t="s">
-        <v>309</v>
-      </c>
-      <c r="G39" s="13" t="s">
-        <v>310</v>
-      </c>
-      <c r="H39" s="13" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="68.099999999999994" customHeight="1">
-      <c r="A40" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="B40" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>311</v>
-      </c>
-      <c r="D40" s="13" t="s">
-        <v>312</v>
-      </c>
-      <c r="E40" s="13" t="s">
-        <v>313</v>
-      </c>
-      <c r="F40" s="13" t="s">
-        <v>314</v>
-      </c>
-      <c r="G40" s="13" t="s">
-        <v>315</v>
-      </c>
       <c r="H40" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A41" s="13" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="G41" s="13" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A42" s="13" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C42" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="E42" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="F42" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="G42" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="H42" s="13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="68.099999999999994" customHeight="1">
+      <c r="A43" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="B43" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>316</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>317</v>
+      </c>
+      <c r="E43" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="F43" s="13" t="s">
+        <v>319</v>
+      </c>
+      <c r="G43" s="13" t="s">
+        <v>320</v>
+      </c>
+      <c r="H43" s="13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="78" customHeight="1">
+      <c r="A44" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="C44" s="13" t="s">
         <v>321</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D44" s="13" t="s">
         <v>322</v>
       </c>
-      <c r="E42" s="13" t="s">
+      <c r="E44" s="13" t="s">
         <v>323</v>
       </c>
-      <c r="F42" s="13" t="s">
+      <c r="F44" s="13" t="s">
         <v>324</v>
       </c>
-      <c r="G42" s="13" t="s">
+      <c r="G44" s="13" t="s">
         <v>325</v>
       </c>
-      <c r="H42" s="13" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="78" customHeight="1">
-      <c r="A43" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B43" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>326</v>
-      </c>
-      <c r="D43" s="13" t="s">
-        <v>327</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>328</v>
-      </c>
-      <c r="F43" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="G43" s="13" t="s">
-        <v>330</v>
-      </c>
-      <c r="H43" s="13" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="68.099999999999994" customHeight="1">
-      <c r="A44" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="C44" s="13" t="s">
-        <v>331</v>
-      </c>
-      <c r="D44" s="13" t="s">
-        <v>332</v>
-      </c>
-      <c r="E44" s="13" t="s">
-        <v>333</v>
-      </c>
-      <c r="F44" s="13" t="s">
-        <v>334</v>
-      </c>
-      <c r="G44" s="13" t="s">
-        <v>335</v>
-      </c>
       <c r="H44" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A45" s="13" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="H45" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A46" s="13" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>343</v>
+        <v>333</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="G46" s="13" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="H46" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A47" s="13" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="G47" s="13" t="s">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A48" s="13" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>351</v>
+        <v>341</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>353</v>
+        <v>343</v>
       </c>
       <c r="F48" s="13" t="s">
-        <v>354</v>
+        <v>344</v>
       </c>
       <c r="G48" s="13" t="s">
-        <v>355</v>
+        <v>345</v>
       </c>
       <c r="H48" s="13" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A49" s="13" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>359</v>
+        <v>349</v>
       </c>
       <c r="G49" s="13" t="s">
-        <v>360</v>
+        <v>350</v>
       </c>
       <c r="H49" s="13" t="s">
-        <v>361</v>
+        <v>190</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A50" s="13" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>363</v>
+        <v>352</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>364</v>
+        <v>353</v>
       </c>
       <c r="F50" s="13" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="G50" s="13" t="s">
-        <v>366</v>
+        <v>355</v>
       </c>
       <c r="H50" s="13" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="68.099999999999994" customHeight="1">
+      <c r="A51" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>357</v>
+      </c>
+      <c r="D51" s="13" t="s">
+        <v>358</v>
+      </c>
+      <c r="E51" s="13" t="s">
+        <v>359</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>360</v>
+      </c>
+      <c r="G51" s="13" t="s">
         <v>361</v>
+      </c>
+      <c r="H51" s="13" t="s">
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: validate application form inputs - Validate required fields, length limits, and application status - Show accessible field errors and preserve invalid input - Revalidate fields with errors as users edit them - Disable browser autocomplete for company and role inputs
</commit_message>
<xml_diff>
--- a/Docs/JobTracker_Development_Tasks.xlsx
+++ b/Docs/JobTracker_Development_Tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Develop\Projects\FrontEnd\job-tracker-fullStack\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1445B38-DC1A-4275-9C71-911833993FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52F75E79-EBBE-4EDB-A3EF-27B433524BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9045" yWindow="2040" windowWidth="28035" windowHeight="16950" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9045" yWindow="255" windowWidth="28035" windowHeight="20220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="任务进度" sheetId="1" r:id="rId1"/>
@@ -32,15 +32,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="397">
   <si>
     <t>Job Tracker 开发任务进度</t>
-  </si>
-  <si>
-    <t>点击 E 列单元格选择状态；仅在验收通过后选择“已验收”。筛选表头可按阶段或状态查看。</t>
-  </si>
-  <si>
-    <t>来源：需求文档 v1.1（第12–27页）及 development-checklist.md；2026-10-04 记录，尚未核实的实现保留待复核。</t>
   </si>
   <si>
     <t>任务数</t>
@@ -1530,11 +1524,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">S0-03 refactor: migrate UI styles to SCSS and organize applications layout
-</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>Order</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -1823,6 +1812,291 @@
         <family val="2"/>
       </rPr>
       <t>scss</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>S0-03 refactor: migrate UI styles to SCSS and organize applications layout
+S0-03 feat: add application modal and unify styles with SCSS
+- Add Sass support and shared design tokens and mixins
+- Migrate component styles to SCSS with BEM naming
+- Move the application form into a reusable Radix UI modal
+- Support form submission through the submit button and Enter key</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>点击</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> E </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>列单元格选择状态；仅在验收通过后选择</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>“</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>已验收</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>。筛选表头可按阶段或状态查看。</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>来源：需求文档</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> v1.1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>（第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>12–27</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>页）及</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> development-checklist.md</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">2026-10-04 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF526579"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>记录，尚未核实的实现保留待复核。</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026.10.10</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>选择</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Linear</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>类似的全局样式</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>引入</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>SCSS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>样式模式
+对应修改每一个组件的样式，包括引入</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>radix-ui</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>用于</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>modal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF223449"/>
+        <rFont val="DengXian"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>封装</t>
     </r>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -1834,7 +2108,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1933,6 +2207,53 @@
       <name val="Calibri"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF526579"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF526579"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF526579"/>
+      <name val="Noto Sans CJK SC"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF526579"/>
+      <name val="DengXian"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF526579"/>
+      <name val="DengXian"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF526579"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF526579"/>
+      <name val="Noto Sans CJK SC"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1970,7 +2291,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2031,6 +2352,12 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2154,8 +2481,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="JobTrackerTasks" displayName="JobTrackerTasks" ref="A7:K53" totalsRowShown="0" dataDxfId="17">
-  <autoFilter ref="A7:K53" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="JobTrackerTasks" displayName="JobTrackerTasks" ref="A6:K52" totalsRowShown="0" dataDxfId="17">
+  <autoFilter ref="A6:K52" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Order" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Stage" dataDxfId="15"/>
@@ -2388,7 +2715,7 @@
   <sheetPr>
     <tabColor rgb="FF243B53"/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="7.125" customWidth="1"/>
@@ -2433,266 +2760,290 @@
       <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11" ht="24" customHeight="1">
-      <c r="A3" s="3" t="s">
-        <v>1</v>
+      <c r="A3" s="21" t="s">
+        <v>393</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="F3" s="22" t="s">
+        <v>394</v>
+      </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" ht="24" customHeight="1">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:11" ht="26.1" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4">
+        <f>COUNTA(C7:C52)</f>
+        <v>46</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" ht="26.1" customHeight="1">
-      <c r="A5" s="4" t="s">
+      <c r="D4" s="4">
+        <f>COUNTIFS(E7:E52,"已验收")</f>
         <v>3</v>
       </c>
-      <c r="B5" s="4">
-        <f>COUNTA(C8:C53)</f>
-        <v>46</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="E4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5">
+        <f>D4/B4</f>
+        <v>6.5217391304347824E-2</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="4">
-        <f>COUNTIFS(E8:E53,"已验收")</f>
-        <v>3</v>
-      </c>
-      <c r="E5" s="4" t="s">
+      <c r="H4" s="4">
+        <f>COUNTIFS(E7:E52,"开发中")</f>
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="5">
-        <f>D5/B5</f>
-        <v>6.5217391304347824E-2</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5" s="4">
-        <f>COUNTIFS(E8:E53,"开发中")</f>
+      <c r="J4" s="4">
+        <f>COUNTIFS(E7:E52,"待复核")</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="4"/>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+    </row>
+    <row r="6" spans="1:11" ht="30" customHeight="1">
+      <c r="A6" s="20" t="s">
+        <v>380</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>381</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>382</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>383</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>384</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>385</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>386</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>388</v>
+      </c>
+      <c r="J6" s="15" t="s">
+        <v>389</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="68.25" customHeight="1">
+      <c r="A7" s="7">
         <v>1</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" s="4">
-        <f>COUNTIFS(E8:E53,"待复核")</f>
-        <v>0</v>
-      </c>
-      <c r="K5" s="4"/>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-    </row>
-    <row r="7" spans="1:11" ht="30" customHeight="1">
-      <c r="A7" s="20" t="s">
-        <v>383</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>384</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>385</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>386</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>387</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>388</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>389</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>390</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>391</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>392</v>
-      </c>
-      <c r="K7" s="20" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="68.25" customHeight="1">
+      <c r="B7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>364</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>363</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="44.1" customHeight="1">
       <c r="A8" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>13</v>
+        <v>378</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="J8" s="16" t="s">
         <v>365</v>
       </c>
       <c r="K8" s="14" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="122.25" customHeight="1">
+      <c r="A9" s="7">
+        <v>3</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="J9" s="16" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="44.1" customHeight="1">
-      <c r="A9" s="7">
-        <v>2</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>364</v>
-      </c>
-      <c r="H9" s="8" t="s">
-        <v>369</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>370</v>
-      </c>
-      <c r="J9" s="16" t="s">
-        <v>367</v>
-      </c>
-      <c r="K9" s="14" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="122.25" customHeight="1">
+      <c r="K9" s="18" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="195" customHeight="1">
       <c r="A10" s="7">
-        <v>3</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>17</v>
+        <v>0</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>375</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>19</v>
+        <v>376</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>377</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>4</v>
       </c>
       <c r="F10" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="J10" s="16" t="s">
+        <v>363</v>
+      </c>
+      <c r="K10" s="18" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="42" customHeight="1">
+      <c r="A11" s="7">
+        <v>4</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="16" t="s">
-        <v>364</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>376</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>374</v>
-      </c>
-      <c r="J10" s="8"/>
-      <c r="K10" s="18" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="122.25" customHeight="1">
-      <c r="A11" s="7">
-        <v>0</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>377</v>
-      </c>
       <c r="C11" s="7" t="s">
-        <v>378</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>379</v>
+        <v>18</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>19</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>380</v>
-      </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="8" t="s">
-        <v>382</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
       <c r="I11" s="9"/>
       <c r="J11" s="8"/>
-      <c r="K11" s="18"/>
+      <c r="K11" s="7" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="12" spans="1:11" ht="42" customHeight="1">
       <c r="A12" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>18</v>
@@ -2702,15 +3053,15 @@
       <c r="I12" s="9"/>
       <c r="J12" s="8"/>
       <c r="K12" s="7" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="42" customHeight="1">
       <c r="A13" s="7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>23</v>
@@ -2719,25 +3070,25 @@
         <v>24</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="9"/>
       <c r="J13" s="8"/>
       <c r="K13" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="42" customHeight="1">
       <c r="A14" s="7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>25</v>
@@ -2746,25 +3097,25 @@
         <v>26</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="9"/>
       <c r="J14" s="8"/>
       <c r="K14" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="42" customHeight="1">
       <c r="A15" s="7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>27</v>
@@ -2773,25 +3124,25 @@
         <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="9"/>
       <c r="J15" s="8"/>
       <c r="K15" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="42" customHeight="1">
       <c r="A16" s="7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>29</v>
@@ -2800,7 +3151,7 @@
         <v>30</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>27</v>
@@ -2810,15 +3161,15 @@
       <c r="I16" s="9"/>
       <c r="J16" s="8"/>
       <c r="K16" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="42" customHeight="1">
       <c r="A17" s="7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>31</v>
@@ -2827,79 +3178,79 @@
         <v>32</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="9"/>
       <c r="J17" s="8"/>
       <c r="K17" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="42" customHeight="1">
       <c r="A18" s="7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G18" s="8"/>
       <c r="H18" s="8"/>
       <c r="I18" s="9"/>
       <c r="J18" s="8"/>
       <c r="K18" s="7" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="42" customHeight="1">
       <c r="A19" s="7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C19" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>39</v>
-      </c>
       <c r="F19" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
       <c r="I19" s="9"/>
       <c r="J19" s="8"/>
       <c r="K19" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="42" customHeight="1">
       <c r="A20" s="7">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>41</v>
@@ -2908,25 +3259,25 @@
         <v>42</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
       <c r="I20" s="9"/>
       <c r="J20" s="8"/>
       <c r="K20" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="42" customHeight="1">
       <c r="A21" s="7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>43</v>
@@ -2935,52 +3286,52 @@
         <v>44</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
       <c r="I21" s="9"/>
       <c r="J21" s="8"/>
       <c r="K21" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="42" customHeight="1">
       <c r="A22" s="7">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
       <c r="I22" s="9"/>
       <c r="J22" s="8"/>
       <c r="K22" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="42" customHeight="1">
       <c r="A23" s="7">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>48</v>
@@ -2989,52 +3340,52 @@
         <v>49</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
       <c r="I23" s="9"/>
       <c r="J23" s="8"/>
       <c r="K23" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="42" customHeight="1">
       <c r="A24" s="7">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
       <c r="I24" s="9"/>
       <c r="J24" s="8"/>
       <c r="K24" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="42" customHeight="1">
       <c r="A25" s="7">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>54</v>
@@ -3043,25 +3394,25 @@
         <v>55</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
       <c r="J25" s="8"/>
       <c r="K25" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="42" customHeight="1">
       <c r="A26" s="7">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>56</v>
@@ -3070,52 +3421,52 @@
         <v>57</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
       <c r="J26" s="8"/>
       <c r="K26" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="42" customHeight="1">
       <c r="A27" s="7">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
       <c r="J27" s="8"/>
       <c r="K27" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="42" customHeight="1">
       <c r="A28" s="7">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>61</v>
@@ -3124,52 +3475,52 @@
         <v>62</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="G28" s="8"/>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
       <c r="J28" s="8"/>
       <c r="K28" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="42" customHeight="1">
       <c r="A29" s="7">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G29" s="8"/>
       <c r="H29" s="8"/>
       <c r="I29" s="9"/>
       <c r="J29" s="8"/>
       <c r="K29" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="42" customHeight="1">
       <c r="A30" s="7">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>66</v>
@@ -3178,52 +3529,52 @@
         <v>67</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
       <c r="I30" s="9"/>
       <c r="J30" s="8"/>
       <c r="K30" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="42" customHeight="1">
       <c r="A31" s="7">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G31" s="8"/>
       <c r="H31" s="8"/>
       <c r="I31" s="9"/>
       <c r="J31" s="8"/>
       <c r="K31" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="42" customHeight="1">
       <c r="A32" s="7">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>72</v>
@@ -3232,25 +3583,25 @@
         <v>73</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G32" s="8"/>
       <c r="H32" s="8"/>
       <c r="I32" s="9"/>
       <c r="J32" s="8"/>
       <c r="K32" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="42" customHeight="1">
       <c r="A33" s="7">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>74</v>
@@ -3259,7 +3610,7 @@
         <v>75</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F33" s="8" t="s">
         <v>72</v>
@@ -3269,15 +3620,15 @@
       <c r="I33" s="9"/>
       <c r="J33" s="8"/>
       <c r="K33" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="42" customHeight="1">
       <c r="A34" s="7">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>76</v>
@@ -3286,7 +3637,7 @@
         <v>77</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>74</v>
@@ -3296,15 +3647,15 @@
       <c r="I34" s="9"/>
       <c r="J34" s="8"/>
       <c r="K34" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="42" customHeight="1">
       <c r="A35" s="7">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>78</v>
@@ -3313,25 +3664,25 @@
         <v>79</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F35" s="8" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G35" s="8"/>
       <c r="H35" s="8"/>
       <c r="I35" s="9"/>
       <c r="J35" s="8"/>
       <c r="K35" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="42" customHeight="1">
       <c r="A36" s="7">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>80</v>
@@ -3340,52 +3691,52 @@
         <v>81</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F36" s="8" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="G36" s="8"/>
       <c r="H36" s="8"/>
       <c r="I36" s="9"/>
       <c r="J36" s="8"/>
       <c r="K36" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="42" customHeight="1">
       <c r="A37" s="7">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F37" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="G37" s="8"/>
       <c r="H37" s="8"/>
       <c r="I37" s="9"/>
       <c r="J37" s="8"/>
       <c r="K37" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="42" customHeight="1">
       <c r="A38" s="7">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C38" s="7" t="s">
         <v>85</v>
@@ -3394,52 +3745,52 @@
         <v>86</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="G38" s="8"/>
       <c r="H38" s="8"/>
       <c r="I38" s="9"/>
       <c r="J38" s="8"/>
       <c r="K38" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="42" customHeight="1">
       <c r="A39" s="7">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F39" s="8" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="G39" s="8"/>
       <c r="H39" s="8"/>
       <c r="I39" s="9"/>
       <c r="J39" s="8"/>
       <c r="K39" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="42" customHeight="1">
       <c r="A40" s="7">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>91</v>
@@ -3448,25 +3799,25 @@
         <v>92</v>
       </c>
       <c r="E40" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="G40" s="8"/>
       <c r="H40" s="8"/>
       <c r="I40" s="9"/>
       <c r="J40" s="8"/>
       <c r="K40" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="42" customHeight="1">
       <c r="A41" s="7">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C41" s="7" t="s">
         <v>93</v>
@@ -3475,7 +3826,7 @@
         <v>94</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F41" s="8" t="s">
         <v>91</v>
@@ -3485,15 +3836,15 @@
       <c r="I41" s="9"/>
       <c r="J41" s="8"/>
       <c r="K41" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="42" customHeight="1">
       <c r="A42" s="7">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C42" s="7" t="s">
         <v>95</v>
@@ -3502,52 +3853,52 @@
         <v>96</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G42" s="8"/>
       <c r="H42" s="8"/>
       <c r="I42" s="9"/>
       <c r="J42" s="8"/>
       <c r="K42" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="42" customHeight="1">
       <c r="A43" s="7">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G43" s="8"/>
       <c r="H43" s="8"/>
       <c r="I43" s="9"/>
       <c r="J43" s="8"/>
       <c r="K43" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="42" customHeight="1">
       <c r="A44" s="7">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C44" s="7" t="s">
         <v>100</v>
@@ -3556,25 +3907,25 @@
         <v>101</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F44" s="8" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G44" s="8"/>
       <c r="H44" s="8"/>
       <c r="I44" s="9"/>
       <c r="J44" s="8"/>
       <c r="K44" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="42" customHeight="1">
       <c r="A45" s="7">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C45" s="7" t="s">
         <v>102</v>
@@ -3583,7 +3934,7 @@
         <v>103</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>100</v>
@@ -3593,15 +3944,15 @@
       <c r="I45" s="9"/>
       <c r="J45" s="8"/>
       <c r="K45" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="42" customHeight="1">
       <c r="A46" s="7">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C46" s="7" t="s">
         <v>104</v>
@@ -3610,79 +3961,79 @@
         <v>105</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F46" s="8" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="G46" s="8"/>
       <c r="H46" s="8"/>
       <c r="I46" s="9"/>
       <c r="J46" s="8"/>
       <c r="K46" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="42" customHeight="1">
       <c r="A47" s="7">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F47" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G47" s="8"/>
       <c r="H47" s="8"/>
       <c r="I47" s="9"/>
       <c r="J47" s="8"/>
       <c r="K47" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="42" customHeight="1">
       <c r="A48" s="7">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
       <c r="I48" s="9"/>
       <c r="J48" s="8"/>
       <c r="K48" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="42" customHeight="1">
       <c r="A49" s="7">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C49" s="7" t="s">
         <v>113</v>
@@ -3691,25 +4042,25 @@
         <v>114</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G49" s="8"/>
       <c r="H49" s="8"/>
       <c r="I49" s="9"/>
       <c r="J49" s="8"/>
       <c r="K49" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="42" customHeight="1">
       <c r="A50" s="7">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C50" s="7" t="s">
         <v>115</v>
@@ -3718,7 +4069,7 @@
         <v>116</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F50" s="8" t="s">
         <v>113</v>
@@ -3728,114 +4079,87 @@
       <c r="I50" s="9"/>
       <c r="J50" s="8"/>
       <c r="K50" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="42" customHeight="1">
       <c r="A51" s="7">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>115</v>
+        <v>66</v>
       </c>
       <c r="G51" s="8"/>
       <c r="H51" s="8"/>
       <c r="I51" s="9"/>
       <c r="J51" s="8"/>
       <c r="K51" s="7" t="s">
-        <v>40</v>
+        <v>121</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="42" customHeight="1">
       <c r="A52" s="7">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C52" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E52" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="D52" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>122</v>
-      </c>
       <c r="F52" s="8" t="s">
-        <v>68</v>
+        <v>104</v>
       </c>
       <c r="G52" s="8"/>
       <c r="H52" s="8"/>
       <c r="I52" s="9"/>
       <c r="J52" s="8"/>
       <c r="K52" s="7" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" ht="42" customHeight="1">
-      <c r="A53" s="7">
-        <v>45</v>
-      </c>
-      <c r="B53" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="E53" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="F53" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="G53" s="8"/>
-      <c r="H53" s="8"/>
-      <c r="I53" s="9"/>
-      <c r="J53" s="8"/>
-      <c r="K53" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="E8:E53">
+  <conditionalFormatting sqref="E7:E52">
     <cfRule type="expression" dxfId="5" priority="1">
-      <formula>$E8="未开始"</formula>
+      <formula>$E7="未开始"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="4" priority="2">
-      <formula>$E8="待复核"</formula>
+      <formula>$E7="待复核"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="3" priority="3">
-      <formula>$E8="开发中"</formula>
+      <formula>$E7="开发中"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="4">
-      <formula>$E8="待验收"</formula>
+      <formula>$E7="待验收"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="5">
-      <formula>$E8="已验收"</formula>
+      <formula>$E7="已验收"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="0" priority="6">
-      <formula>$E8="暂缓"</formula>
+      <formula>$E7="暂缓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="E8:E53" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="E7:E52" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"未开始,待复核,开发中,待验收,已验收,暂缓"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3876,7 +4200,7 @@
     </row>
     <row r="2" spans="1:8" ht="27.95" customHeight="1">
       <c r="A2" s="11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -3888,7 +4212,7 @@
     </row>
     <row r="3" spans="1:8" ht="24" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
@@ -3900,7 +4224,7 @@
     </row>
     <row r="4" spans="1:8" ht="24" customHeight="1">
       <c r="A4" s="12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -3912,93 +4236,93 @@
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>132</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A6" s="13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="D6" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="F6" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="G6" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="F6" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>138</v>
-      </c>
       <c r="H6" s="17" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A7" s="13" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C7" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="E7" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="F7" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="G7" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="F7" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>144</v>
-      </c>
       <c r="H7" s="13" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="112.5" customHeight="1">
       <c r="A8" s="13" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
       <c r="E8" s="13" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
@@ -4006,1120 +4330,1120 @@
     </row>
     <row r="9" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C9" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="F9" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="G9" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="E9" s="13" t="s">
-        <v>373</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>148</v>
-      </c>
       <c r="H9" s="13" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A10" s="13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C10" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="E10" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="F10" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="G10" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="H10" s="13" t="s">
         <v>152</v>
-      </c>
-      <c r="G10" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="H10" s="13" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A11" s="13" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C11" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="E11" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="F11" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="G11" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="F11" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>159</v>
-      </c>
       <c r="H11" s="13" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C12" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="E12" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="F12" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="G12" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="F12" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>164</v>
-      </c>
       <c r="H12" s="13" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A13" s="13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C13" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="E13" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="F13" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="G13" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="F13" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>169</v>
-      </c>
       <c r="H13" s="13" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A14" s="13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C14" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="E14" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="F14" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="G14" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="F14" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="G14" s="13" t="s">
-        <v>174</v>
-      </c>
       <c r="H14" s="13" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C15" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="E15" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="F15" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="G15" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="F15" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="G15" s="13" t="s">
-        <v>179</v>
-      </c>
       <c r="H15" s="13" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A16" s="13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C16" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="E16" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="F16" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="G16" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="F16" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>184</v>
-      </c>
       <c r="H16" s="13" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A17" s="13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C17" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="E17" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="F17" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="G17" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="F17" s="13" t="s">
+      <c r="H17" s="13" t="s">
         <v>188</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A18" s="13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C18" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="E18" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="F18" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="G18" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="F18" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>195</v>
-      </c>
       <c r="H18" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A19" s="13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C19" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="E19" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="F19" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="G19" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="F19" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>200</v>
-      </c>
       <c r="H19" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A20" s="13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C20" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="E20" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="F20" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="G20" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="F20" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="G20" s="13" t="s">
-        <v>205</v>
-      </c>
       <c r="H20" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C21" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="E21" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="F21" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="G21" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="F21" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>210</v>
-      </c>
       <c r="H21" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A22" s="13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C22" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="E22" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="F22" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="G22" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="F22" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="G22" s="13" t="s">
-        <v>215</v>
-      </c>
       <c r="H22" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A23" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C23" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="E23" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="F23" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="G23" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="F23" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="G23" s="13" t="s">
-        <v>220</v>
-      </c>
       <c r="H23" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A24" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C24" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="E24" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="F24" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="G24" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="F24" s="13" t="s">
-        <v>224</v>
-      </c>
-      <c r="G24" s="13" t="s">
-        <v>225</v>
-      </c>
       <c r="H24" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C25" s="13" t="s">
+        <v>224</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="E25" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="F25" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="G25" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="F25" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="G25" s="13" t="s">
-        <v>230</v>
-      </c>
       <c r="H25" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A26" s="13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C26" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="E26" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="F26" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="G26" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="F26" s="13" t="s">
-        <v>234</v>
-      </c>
-      <c r="G26" s="13" t="s">
-        <v>235</v>
-      </c>
       <c r="H26" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A27" s="13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C27" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="E27" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="F27" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="E27" s="13" t="s">
+      <c r="G27" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="F27" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>240</v>
-      </c>
       <c r="H27" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A28" s="13" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C28" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="E28" s="13" t="s">
         <v>241</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="F28" s="13" t="s">
         <v>242</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="G28" s="13" t="s">
         <v>243</v>
       </c>
-      <c r="F28" s="13" t="s">
-        <v>244</v>
-      </c>
-      <c r="G28" s="13" t="s">
-        <v>245</v>
-      </c>
       <c r="H28" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C29" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="E29" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="F29" s="13" t="s">
         <v>247</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="G29" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="F29" s="13" t="s">
-        <v>249</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>250</v>
-      </c>
       <c r="H29" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A30" s="13" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C30" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="E30" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="F30" s="13" t="s">
         <v>252</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="G30" s="13" t="s">
         <v>253</v>
       </c>
-      <c r="F30" s="13" t="s">
-        <v>254</v>
-      </c>
-      <c r="G30" s="13" t="s">
-        <v>255</v>
-      </c>
       <c r="H30" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A31" s="13" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C31" s="13" t="s">
+        <v>254</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>255</v>
+      </c>
+      <c r="E31" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="F31" s="13" t="s">
         <v>257</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="G31" s="13" t="s">
         <v>258</v>
       </c>
-      <c r="F31" s="13" t="s">
-        <v>259</v>
-      </c>
-      <c r="G31" s="13" t="s">
-        <v>260</v>
-      </c>
       <c r="H31" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A32" s="13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C32" s="13" t="s">
+        <v>259</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>260</v>
+      </c>
+      <c r="E32" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="D32" s="13" t="s">
+      <c r="F32" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="E32" s="13" t="s">
+      <c r="G32" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="F32" s="13" t="s">
-        <v>264</v>
-      </c>
-      <c r="G32" s="13" t="s">
-        <v>265</v>
-      </c>
       <c r="H32" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A33" s="13" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C33" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="E33" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="D33" s="13" t="s">
+      <c r="F33" s="13" t="s">
         <v>267</v>
       </c>
-      <c r="E33" s="13" t="s">
+      <c r="G33" s="13" t="s">
         <v>268</v>
       </c>
-      <c r="F33" s="13" t="s">
-        <v>269</v>
-      </c>
-      <c r="G33" s="13" t="s">
-        <v>270</v>
-      </c>
       <c r="H33" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A34" s="13" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C34" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="E34" s="13" t="s">
         <v>271</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="F34" s="13" t="s">
         <v>272</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="G34" s="13" t="s">
         <v>273</v>
       </c>
-      <c r="F34" s="13" t="s">
-        <v>274</v>
-      </c>
-      <c r="G34" s="13" t="s">
-        <v>275</v>
-      </c>
       <c r="H34" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C35" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="E35" s="13" t="s">
         <v>276</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="F35" s="13" t="s">
         <v>277</v>
       </c>
-      <c r="E35" s="13" t="s">
+      <c r="G35" s="13" t="s">
         <v>278</v>
       </c>
-      <c r="F35" s="13" t="s">
-        <v>279</v>
-      </c>
-      <c r="G35" s="13" t="s">
-        <v>280</v>
-      </c>
       <c r="H35" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A36" s="13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C36" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="E36" s="13" t="s">
         <v>281</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="F36" s="13" t="s">
         <v>282</v>
       </c>
-      <c r="E36" s="13" t="s">
+      <c r="G36" s="13" t="s">
         <v>283</v>
       </c>
-      <c r="F36" s="13" t="s">
-        <v>284</v>
-      </c>
-      <c r="G36" s="13" t="s">
-        <v>285</v>
-      </c>
       <c r="H36" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A37" s="13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C37" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="E37" s="13" t="s">
         <v>286</v>
       </c>
-      <c r="D37" s="13" t="s">
+      <c r="F37" s="13" t="s">
         <v>287</v>
       </c>
-      <c r="E37" s="13" t="s">
+      <c r="G37" s="13" t="s">
         <v>288</v>
       </c>
-      <c r="F37" s="13" t="s">
-        <v>289</v>
-      </c>
-      <c r="G37" s="13" t="s">
-        <v>290</v>
-      </c>
       <c r="H37" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A38" s="13" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C38" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="E38" s="13" t="s">
         <v>291</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="F38" s="13" t="s">
         <v>292</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="G38" s="13" t="s">
         <v>293</v>
       </c>
-      <c r="F38" s="13" t="s">
-        <v>294</v>
-      </c>
-      <c r="G38" s="13" t="s">
-        <v>295</v>
-      </c>
       <c r="H38" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A39" s="13" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C39" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="E39" s="13" t="s">
         <v>296</v>
       </c>
-      <c r="D39" s="13" t="s">
+      <c r="F39" s="13" t="s">
         <v>297</v>
       </c>
-      <c r="E39" s="13" t="s">
+      <c r="G39" s="13" t="s">
         <v>298</v>
       </c>
-      <c r="F39" s="13" t="s">
-        <v>299</v>
-      </c>
-      <c r="G39" s="13" t="s">
-        <v>300</v>
-      </c>
       <c r="H39" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="78" customHeight="1">
       <c r="A40" s="13" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C40" s="13" t="s">
+        <v>299</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="E40" s="13" t="s">
         <v>301</v>
       </c>
-      <c r="D40" s="13" t="s">
+      <c r="F40" s="13" t="s">
         <v>302</v>
       </c>
-      <c r="E40" s="13" t="s">
+      <c r="G40" s="13" t="s">
         <v>303</v>
       </c>
-      <c r="F40" s="13" t="s">
-        <v>304</v>
-      </c>
-      <c r="G40" s="13" t="s">
-        <v>305</v>
-      </c>
       <c r="H40" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A41" s="13" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C41" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="E41" s="13" t="s">
         <v>306</v>
       </c>
-      <c r="D41" s="13" t="s">
+      <c r="F41" s="13" t="s">
         <v>307</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="G41" s="13" t="s">
         <v>308</v>
       </c>
-      <c r="F41" s="13" t="s">
-        <v>309</v>
-      </c>
-      <c r="G41" s="13" t="s">
-        <v>310</v>
-      </c>
       <c r="H41" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A42" s="13" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C42" s="13" t="s">
+        <v>309</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>310</v>
+      </c>
+      <c r="E42" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="F42" s="13" t="s">
         <v>312</v>
       </c>
-      <c r="E42" s="13" t="s">
+      <c r="G42" s="13" t="s">
         <v>313</v>
       </c>
-      <c r="F42" s="13" t="s">
-        <v>314</v>
-      </c>
-      <c r="G42" s="13" t="s">
-        <v>315</v>
-      </c>
       <c r="H42" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A43" s="13" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C43" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="E43" s="13" t="s">
         <v>316</v>
       </c>
-      <c r="D43" s="13" t="s">
+      <c r="F43" s="13" t="s">
         <v>317</v>
       </c>
-      <c r="E43" s="13" t="s">
+      <c r="G43" s="13" t="s">
         <v>318</v>
       </c>
-      <c r="F43" s="13" t="s">
-        <v>319</v>
-      </c>
-      <c r="G43" s="13" t="s">
-        <v>320</v>
-      </c>
       <c r="H43" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="78" customHeight="1">
       <c r="A44" s="13" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C44" s="13" t="s">
+        <v>319</v>
+      </c>
+      <c r="D44" s="13" t="s">
+        <v>320</v>
+      </c>
+      <c r="E44" s="13" t="s">
         <v>321</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="F44" s="13" t="s">
         <v>322</v>
       </c>
-      <c r="E44" s="13" t="s">
+      <c r="G44" s="13" t="s">
         <v>323</v>
       </c>
-      <c r="F44" s="13" t="s">
-        <v>324</v>
-      </c>
-      <c r="G44" s="13" t="s">
-        <v>325</v>
-      </c>
       <c r="H44" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A45" s="13" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C45" s="13" t="s">
+        <v>324</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>325</v>
+      </c>
+      <c r="E45" s="13" t="s">
         <v>326</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="F45" s="13" t="s">
         <v>327</v>
       </c>
-      <c r="E45" s="13" t="s">
+      <c r="G45" s="13" t="s">
         <v>328</v>
       </c>
-      <c r="F45" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="G45" s="13" t="s">
-        <v>330</v>
-      </c>
       <c r="H45" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A46" s="13" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C46" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="D46" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="E46" s="13" t="s">
         <v>331</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="F46" s="13" t="s">
         <v>332</v>
       </c>
-      <c r="E46" s="13" t="s">
+      <c r="G46" s="13" t="s">
         <v>333</v>
       </c>
-      <c r="F46" s="13" t="s">
-        <v>334</v>
-      </c>
-      <c r="G46" s="13" t="s">
-        <v>335</v>
-      </c>
       <c r="H46" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A47" s="13" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C47" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="D47" s="13" t="s">
+        <v>335</v>
+      </c>
+      <c r="E47" s="13" t="s">
         <v>336</v>
       </c>
-      <c r="D47" s="13" t="s">
+      <c r="F47" s="13" t="s">
         <v>337</v>
       </c>
-      <c r="E47" s="13" t="s">
+      <c r="G47" s="13" t="s">
         <v>338</v>
       </c>
-      <c r="F47" s="13" t="s">
-        <v>339</v>
-      </c>
-      <c r="G47" s="13" t="s">
-        <v>340</v>
-      </c>
       <c r="H47" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A48" s="13" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C48" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="D48" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="E48" s="13" t="s">
         <v>341</v>
       </c>
-      <c r="D48" s="13" t="s">
+      <c r="F48" s="13" t="s">
         <v>342</v>
       </c>
-      <c r="E48" s="13" t="s">
+      <c r="G48" s="13" t="s">
         <v>343</v>
       </c>
-      <c r="F48" s="13" t="s">
-        <v>344</v>
-      </c>
-      <c r="G48" s="13" t="s">
-        <v>345</v>
-      </c>
       <c r="H48" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A49" s="13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C49" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="D49" s="13" t="s">
+        <v>345</v>
+      </c>
+      <c r="E49" s="13" t="s">
         <v>346</v>
       </c>
-      <c r="D49" s="13" t="s">
+      <c r="F49" s="13" t="s">
         <v>347</v>
       </c>
-      <c r="E49" s="13" t="s">
+      <c r="G49" s="13" t="s">
         <v>348</v>
       </c>
-      <c r="F49" s="13" t="s">
-        <v>349</v>
-      </c>
-      <c r="G49" s="13" t="s">
-        <v>350</v>
-      </c>
       <c r="H49" s="13" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A50" s="13" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C50" s="13" t="s">
+        <v>349</v>
+      </c>
+      <c r="D50" s="13" t="s">
+        <v>350</v>
+      </c>
+      <c r="E50" s="13" t="s">
         <v>351</v>
       </c>
-      <c r="D50" s="13" t="s">
+      <c r="F50" s="13" t="s">
         <v>352</v>
       </c>
-      <c r="E50" s="13" t="s">
+      <c r="G50" s="13" t="s">
         <v>353</v>
       </c>
-      <c r="F50" s="13" t="s">
+      <c r="H50" s="13" t="s">
         <v>354</v>
-      </c>
-      <c r="G50" s="13" t="s">
-        <v>355</v>
-      </c>
-      <c r="H50" s="13" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="68.099999999999994" customHeight="1">
       <c r="A51" s="13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C51" s="13" t="s">
+        <v>355</v>
+      </c>
+      <c r="D51" s="13" t="s">
+        <v>356</v>
+      </c>
+      <c r="E51" s="13" t="s">
         <v>357</v>
       </c>
-      <c r="D51" s="13" t="s">
+      <c r="F51" s="13" t="s">
         <v>358</v>
       </c>
-      <c r="E51" s="13" t="s">
+      <c r="G51" s="13" t="s">
         <v>359</v>
       </c>
-      <c r="F51" s="13" t="s">
-        <v>360</v>
-      </c>
-      <c r="G51" s="13" t="s">
-        <v>361</v>
-      </c>
       <c r="H51" s="13" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>